<commit_message>
Improve testbench validation and DQ60 point selection
</commit_message>
<xml_diff>
--- a/01_自吸方案/02_台架测试_10kW/04_验证结果/CEGR_testbench_visualization_results.xlsx
+++ b/01_自吸方案/02_台架测试_10kW/04_验证结果/CEGR_testbench_visualization_results.xlsx
@@ -11,13 +11,16 @@
     <sheet name="constant_pO2_DQ60_two_point" sheetId="3" r:id="rId5"/>
     <sheet name="constant_pO2_DQ60_comparison" sheetId="4" r:id="rId6"/>
     <sheet name="run_info" sheetId="5" r:id="rId7"/>
+    <sheet name="no_egr_validation" sheetId="6" r:id="rId8"/>
+    <sheet name="no_egr_validation_stats" sheetId="7" r:id="rId9"/>
+    <sheet name="topology_case" sheetId="8" r:id="rId10"/>
   </sheets>
   <calcPr calcId="125725" fullCalcOnLoad="true"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="1418" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="7076" uniqueCount="194">
   <si>
     <t>condition</t>
   </si>
@@ -458,6 +461,147 @@
   </si>
   <si>
     <t>2026-06-07 13:35:09</t>
+  </si>
+  <si>
+    <t>case_index</t>
+  </si>
+  <si>
+    <t>bench_152A</t>
+  </si>
+  <si>
+    <t>bench_228A</t>
+  </si>
+  <si>
+    <t>bench_266A</t>
+  </si>
+  <si>
+    <t>bench_342A</t>
+  </si>
+  <si>
+    <t>bench_418A</t>
+  </si>
+  <si>
+    <t>bench_494A</t>
+  </si>
+  <si>
+    <t>bench_570A</t>
+  </si>
+  <si>
+    <t>bench_646A</t>
+  </si>
+  <si>
+    <t>bench_684A</t>
+  </si>
+  <si>
+    <t>bench_722A</t>
+  </si>
+  <si>
+    <t>V_cell_bench</t>
+  </si>
+  <si>
+    <t>T_stack_fit_C</t>
+  </si>
+  <si>
+    <t>cathode_in_pressure_abs_kPa</t>
+  </si>
+  <si>
+    <t>cathode_RH</t>
+  </si>
+  <si>
+    <t>V_cell_err</t>
+  </si>
+  <si>
+    <t>T_stack_err_C</t>
+  </si>
+  <si>
+    <t>p_ca_in_err_kPa</t>
+  </si>
+  <si>
+    <t>RH_ca_in_err</t>
+  </si>
+  <si>
+    <t>metric</t>
+  </si>
+  <si>
+    <t>rmse</t>
+  </si>
+  <si>
+    <t>max_abs_error</t>
+  </si>
+  <si>
+    <t>point_count</t>
+  </si>
+  <si>
+    <t>2026-06-07 13:47:15</t>
+  </si>
+  <si>
+    <t>2026-06-07 13:56:38</t>
+  </si>
+  <si>
+    <t>lambda_O2_final_sample</t>
+  </si>
+  <si>
+    <t>lambda_O2_window_min</t>
+  </si>
+  <si>
+    <t>lambda_O2_window_max</t>
+  </si>
+  <si>
+    <t>lambda_O2_window_range</t>
+  </si>
+  <si>
+    <t>m_ca_in_actual_kg_s</t>
+  </si>
+  <si>
+    <t>m_ca_in_final_sample_kg_s</t>
+  </si>
+  <si>
+    <t>ca_in_flowing_fraction_30s</t>
+  </si>
+  <si>
+    <t>dV_cell_30s</t>
+  </si>
+  <si>
+    <t>dp_stack_internal_30s_kPa</t>
+  </si>
+  <si>
+    <t>is_dynamic_stable</t>
+  </si>
+  <si>
+    <t>coarse_grid</t>
+  </si>
+  <si>
+    <t>dynamic_oscillation</t>
+  </si>
+  <si>
+    <t>2026-06-07 14:16:22</t>
+  </si>
+  <si>
+    <t>2026-06-07 14:33:18</t>
+  </si>
+  <si>
+    <t>2026-06-07 14:36:44</t>
+  </si>
+  <si>
+    <t>representative_j0p10_EGR0p25_DQ60_solved_min_stable_flow</t>
+  </si>
+  <si>
+    <t>best_effort_unreachable_with_DQ60_map</t>
+  </si>
+  <si>
+    <t>two_point_solved_min_stable_DQ60_flow</t>
+  </si>
+  <si>
+    <t>selection_score</t>
+  </si>
+  <si>
+    <t>pO2_target_miss</t>
+  </si>
+  <si>
+    <t>2026-06-07 15:00:36</t>
+  </si>
+  <si>
+    <t>2026-06-07 15:12:31</t>
   </si>
 </sst>
 </file>
@@ -13021,7 +13165,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:BS3"/>
+  <dimension ref="A1:CD3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="27.44140625" customWidth="true"/>
@@ -13045,56 +13189,67 @@
     <col min="19" max="19" width="11.5546875" customWidth="true"/>
     <col min="20" max="20" width="11.5546875" customWidth="true"/>
     <col min="21" max="21" width="16.33203125" customWidth="true"/>
-    <col min="22" max="22" width="18.5546875" customWidth="true"/>
-    <col min="23" max="23" width="16.6640625" customWidth="true"/>
-    <col min="24" max="24" width="16.77734375" customWidth="true"/>
-    <col min="25" max="25" width="19.6640625" customWidth="true"/>
-    <col min="26" max="26" width="15.77734375" customWidth="true"/>
-    <col min="27" max="27" width="15" customWidth="true"/>
-    <col min="28" max="28" width="13.6640625" customWidth="true"/>
-    <col min="29" max="29" width="11.88671875" customWidth="true"/>
-    <col min="30" max="30" width="17.77734375" customWidth="true"/>
-    <col min="31" max="31" width="14" customWidth="true"/>
-    <col min="32" max="32" width="22.109375" customWidth="true"/>
-    <col min="33" max="33" width="13.33203125" customWidth="true"/>
-    <col min="34" max="34" width="11.5546875" customWidth="true"/>
-    <col min="35" max="35" width="14.6640625" customWidth="true"/>
-    <col min="36" max="36" width="12.88671875" customWidth="true"/>
-    <col min="37" max="37" width="9.44140625" customWidth="true"/>
-    <col min="38" max="38" width="11.21875" customWidth="true"/>
-    <col min="39" max="39" width="11.5546875" customWidth="true"/>
-    <col min="40" max="40" width="13.5546875" customWidth="true"/>
-    <col min="41" max="41" width="8.6640625" customWidth="true"/>
-    <col min="42" max="42" width="13" customWidth="true"/>
-    <col min="43" max="43" width="23.88671875" customWidth="true"/>
-    <col min="44" max="44" width="17.77734375" customWidth="true"/>
-    <col min="45" max="45" width="19.109375" customWidth="true"/>
-    <col min="46" max="46" width="20.44140625" customWidth="true"/>
-    <col min="47" max="47" width="19.5546875" customWidth="true"/>
-    <col min="48" max="48" width="18.44140625" customWidth="true"/>
-    <col min="49" max="49" width="15.5546875" customWidth="true"/>
-    <col min="50" max="50" width="14.5546875" customWidth="true"/>
-    <col min="51" max="51" width="26.109375" customWidth="true"/>
-    <col min="52" max="52" width="20" customWidth="true"/>
-    <col min="53" max="53" width="19.44140625" customWidth="true"/>
-    <col min="54" max="54" width="24.5546875" customWidth="true"/>
-    <col min="55" max="55" width="17.109375" customWidth="true"/>
-    <col min="56" max="56" width="16.33203125" customWidth="true"/>
-    <col min="57" max="57" width="23.44140625" customWidth="true"/>
-    <col min="58" max="58" width="23.88671875" customWidth="true"/>
-    <col min="59" max="59" width="21.88671875" customWidth="true"/>
-    <col min="60" max="60" width="38" customWidth="true"/>
-    <col min="61" max="61" width="13" customWidth="true"/>
-    <col min="62" max="62" width="28.44140625" customWidth="true"/>
-    <col min="63" max="63" width="13.21875" customWidth="true"/>
-    <col min="64" max="64" width="9.77734375" customWidth="true"/>
-    <col min="65" max="65" width="10.33203125" customWidth="true"/>
-    <col min="66" max="66" width="11" customWidth="true"/>
-    <col min="67" max="67" width="18.44140625" customWidth="true"/>
-    <col min="68" max="68" width="21.33203125" customWidth="true"/>
-    <col min="69" max="69" width="18.77734375" customWidth="true"/>
-    <col min="70" max="70" width="18.21875" customWidth="true"/>
-    <col min="71" max="71" width="18.21875" customWidth="true"/>
+    <col min="22" max="22" width="21.6640625" customWidth="true"/>
+    <col min="23" max="23" width="21.77734375" customWidth="true"/>
+    <col min="24" max="24" width="22.21875" customWidth="true"/>
+    <col min="25" max="25" width="23.33203125" customWidth="true"/>
+    <col min="26" max="26" width="18.44140625" customWidth="true"/>
+    <col min="27" max="27" width="23.77734375" customWidth="true"/>
+    <col min="28" max="28" width="23.5546875" customWidth="true"/>
+    <col min="29" max="29" width="15.5546875" customWidth="true"/>
+    <col min="30" max="30" width="23.109375" customWidth="true"/>
+    <col min="31" max="31" width="15.88671875" customWidth="true"/>
+    <col min="32" max="32" width="18.5546875" customWidth="true"/>
+    <col min="33" max="33" width="16.6640625" customWidth="true"/>
+    <col min="34" max="34" width="16.77734375" customWidth="true"/>
+    <col min="35" max="35" width="19.6640625" customWidth="true"/>
+    <col min="36" max="36" width="15.77734375" customWidth="true"/>
+    <col min="37" max="37" width="15" customWidth="true"/>
+    <col min="38" max="38" width="13.6640625" customWidth="true"/>
+    <col min="39" max="39" width="11.88671875" customWidth="true"/>
+    <col min="40" max="40" width="17.77734375" customWidth="true"/>
+    <col min="41" max="41" width="14" customWidth="true"/>
+    <col min="42" max="42" width="22.109375" customWidth="true"/>
+    <col min="43" max="43" width="13.33203125" customWidth="true"/>
+    <col min="44" max="44" width="11.5546875" customWidth="true"/>
+    <col min="45" max="45" width="14.6640625" customWidth="true"/>
+    <col min="46" max="46" width="12.88671875" customWidth="true"/>
+    <col min="47" max="47" width="9.44140625" customWidth="true"/>
+    <col min="48" max="48" width="11.21875" customWidth="true"/>
+    <col min="49" max="49" width="11.5546875" customWidth="true"/>
+    <col min="50" max="50" width="13.5546875" customWidth="true"/>
+    <col min="51" max="51" width="8.6640625" customWidth="true"/>
+    <col min="52" max="52" width="13" customWidth="true"/>
+    <col min="53" max="53" width="23.88671875" customWidth="true"/>
+    <col min="54" max="54" width="17.77734375" customWidth="true"/>
+    <col min="55" max="55" width="19.109375" customWidth="true"/>
+    <col min="56" max="56" width="20.44140625" customWidth="true"/>
+    <col min="57" max="57" width="19.5546875" customWidth="true"/>
+    <col min="58" max="58" width="18.44140625" customWidth="true"/>
+    <col min="59" max="59" width="15.5546875" customWidth="true"/>
+    <col min="60" max="60" width="14.5546875" customWidth="true"/>
+    <col min="61" max="61" width="26.109375" customWidth="true"/>
+    <col min="62" max="62" width="20" customWidth="true"/>
+    <col min="63" max="63" width="19.44140625" customWidth="true"/>
+    <col min="64" max="64" width="24.5546875" customWidth="true"/>
+    <col min="65" max="65" width="17.109375" customWidth="true"/>
+    <col min="66" max="66" width="16.33203125" customWidth="true"/>
+    <col min="67" max="67" width="23.44140625" customWidth="true"/>
+    <col min="68" max="68" width="23.88671875" customWidth="true"/>
+    <col min="69" max="69" width="21.88671875" customWidth="true"/>
+    <col min="70" max="70" width="35.77734375" customWidth="true"/>
+    <col min="71" max="71" width="13" customWidth="true"/>
+    <col min="72" max="72" width="10.33203125" customWidth="true"/>
+    <col min="73" max="73" width="11" customWidth="true"/>
+    <col min="74" max="74" width="13.21875" customWidth="true"/>
+    <col min="75" max="75" width="9.77734375" customWidth="true"/>
+    <col min="76" max="76" width="21.33203125" customWidth="true"/>
+    <col min="77" max="77" width="13.77734375" customWidth="true"/>
+    <col min="78" max="78" width="28.44140625" customWidth="true"/>
+    <col min="79" max="79" width="18.44140625" customWidth="true"/>
+    <col min="80" max="80" width="18.77734375" customWidth="true"/>
+    <col min="81" max="81" width="18.21875" customWidth="true"/>
+    <col min="82" max="82" width="18.21875" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -13162,153 +13317,186 @@
         <v>24</v>
       </c>
       <c r="V1" s="0" t="s">
+        <v>172</v>
+      </c>
+      <c r="W1" s="0" t="s">
+        <v>173</v>
+      </c>
+      <c r="X1" s="0" t="s">
+        <v>174</v>
+      </c>
+      <c r="Y1" s="0" t="s">
+        <v>175</v>
+      </c>
+      <c r="Z1" s="0" t="s">
+        <v>176</v>
+      </c>
+      <c r="AA1" s="0" t="s">
+        <v>177</v>
+      </c>
+      <c r="AB1" s="0" t="s">
+        <v>178</v>
+      </c>
+      <c r="AC1" s="0" t="s">
+        <v>179</v>
+      </c>
+      <c r="AD1" s="0" t="s">
+        <v>180</v>
+      </c>
+      <c r="AE1" s="0" t="s">
+        <v>181</v>
+      </c>
+      <c r="AF1" s="0" t="s">
         <v>25</v>
       </c>
-      <c r="W1" s="0" t="s">
+      <c r="AG1" s="0" t="s">
         <v>26</v>
       </c>
-      <c r="X1" s="0" t="s">
+      <c r="AH1" s="0" t="s">
         <v>27</v>
       </c>
-      <c r="Y1" s="0" t="s">
+      <c r="AI1" s="0" t="s">
         <v>28</v>
       </c>
-      <c r="Z1" s="0" t="s">
+      <c r="AJ1" s="0" t="s">
         <v>29</v>
       </c>
-      <c r="AA1" s="0" t="s">
+      <c r="AK1" s="0" t="s">
         <v>30</v>
       </c>
-      <c r="AB1" s="0" t="s">
+      <c r="AL1" s="0" t="s">
         <v>31</v>
       </c>
-      <c r="AC1" s="0" t="s">
+      <c r="AM1" s="0" t="s">
         <v>32</v>
       </c>
-      <c r="AD1" s="0" t="s">
+      <c r="AN1" s="0" t="s">
         <v>33</v>
       </c>
-      <c r="AE1" s="0" t="s">
+      <c r="AO1" s="0" t="s">
         <v>34</v>
       </c>
-      <c r="AF1" s="0" t="s">
+      <c r="AP1" s="0" t="s">
         <v>35</v>
       </c>
-      <c r="AG1" s="0" t="s">
+      <c r="AQ1" s="0" t="s">
         <v>36</v>
       </c>
-      <c r="AH1" s="0" t="s">
+      <c r="AR1" s="0" t="s">
         <v>37</v>
       </c>
-      <c r="AI1" s="0" t="s">
+      <c r="AS1" s="0" t="s">
         <v>38</v>
       </c>
-      <c r="AJ1" s="0" t="s">
+      <c r="AT1" s="0" t="s">
         <v>39</v>
       </c>
-      <c r="AK1" s="0" t="s">
+      <c r="AU1" s="0" t="s">
         <v>40</v>
       </c>
-      <c r="AL1" s="0" t="s">
+      <c r="AV1" s="0" t="s">
         <v>41</v>
       </c>
-      <c r="AM1" s="0" t="s">
+      <c r="AW1" s="0" t="s">
         <v>42</v>
       </c>
-      <c r="AN1" s="0" t="s">
+      <c r="AX1" s="0" t="s">
         <v>43</v>
       </c>
-      <c r="AO1" s="0" t="s">
+      <c r="AY1" s="0" t="s">
         <v>44</v>
       </c>
-      <c r="AP1" s="0" t="s">
+      <c r="AZ1" s="0" t="s">
         <v>45</v>
       </c>
-      <c r="AQ1" s="0" t="s">
+      <c r="BA1" s="0" t="s">
         <v>46</v>
       </c>
-      <c r="AR1" s="0" t="s">
+      <c r="BB1" s="0" t="s">
         <v>47</v>
       </c>
-      <c r="AS1" s="0" t="s">
+      <c r="BC1" s="0" t="s">
         <v>48</v>
       </c>
-      <c r="AT1" s="0" t="s">
+      <c r="BD1" s="0" t="s">
         <v>49</v>
       </c>
-      <c r="AU1" s="0" t="s">
+      <c r="BE1" s="0" t="s">
         <v>50</v>
       </c>
-      <c r="AV1" s="0" t="s">
+      <c r="BF1" s="0" t="s">
         <v>84</v>
       </c>
-      <c r="AW1" s="0" t="s">
+      <c r="BG1" s="0" t="s">
         <v>87</v>
       </c>
-      <c r="AX1" s="0" t="s">
+      <c r="BH1" s="0" t="s">
         <v>74</v>
       </c>
-      <c r="AY1" s="0" t="s">
+      <c r="BI1" s="0" t="s">
         <v>51</v>
       </c>
-      <c r="AZ1" s="0" t="s">
+      <c r="BJ1" s="0" t="s">
         <v>91</v>
       </c>
-      <c r="BA1" s="0" t="s">
+      <c r="BK1" s="0" t="s">
         <v>92</v>
       </c>
-      <c r="BB1" s="0" t="s">
+      <c r="BL1" s="0" t="s">
         <v>93</v>
       </c>
-      <c r="BC1" s="0" t="s">
+      <c r="BM1" s="0" t="s">
         <v>94</v>
       </c>
-      <c r="BD1" s="0" t="s">
+      <c r="BN1" s="0" t="s">
         <v>58</v>
       </c>
-      <c r="BE1" s="0" t="s">
+      <c r="BO1" s="0" t="s">
         <v>95</v>
       </c>
-      <c r="BF1" s="0" t="s">
+      <c r="BP1" s="0" t="s">
         <v>96</v>
       </c>
-      <c r="BG1" s="0" t="s">
+      <c r="BQ1" s="0" t="s">
         <v>97</v>
       </c>
-      <c r="BH1" s="0" t="s">
+      <c r="BR1" s="0" t="s">
         <v>52</v>
       </c>
-      <c r="BI1" s="0" t="s">
+      <c r="BS1" s="0" t="s">
         <v>80</v>
       </c>
-      <c r="BJ1" s="0" t="s">
+      <c r="BT1" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="BU1" s="0" t="s">
+        <v>57</v>
+      </c>
+      <c r="BV1" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="BW1" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="BX1" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="BY1" s="0" t="s">
+        <v>190</v>
+      </c>
+      <c r="BZ1" s="0" t="s">
         <v>54</v>
       </c>
-      <c r="BK1" s="0" t="s">
-        <v>100</v>
-      </c>
-      <c r="BL1" s="0" t="s">
-        <v>55</v>
-      </c>
-      <c r="BM1" s="0" t="s">
-        <v>56</v>
-      </c>
-      <c r="BN1" s="0" t="s">
-        <v>57</v>
-      </c>
-      <c r="BO1" s="0" t="s">
+      <c r="CA1" s="0" t="s">
         <v>101</v>
       </c>
-      <c r="BP1" s="0" t="s">
-        <v>102</v>
-      </c>
-      <c r="BQ1" s="0" t="s">
+      <c r="CB1" s="0" t="s">
         <v>60</v>
       </c>
-      <c r="BR1" s="0" t="s">
+      <c r="CC1" s="0" t="s">
         <v>61</v>
       </c>
-      <c r="BS1" s="0" t="s">
+      <c r="CD1" s="0" t="s">
         <v>64</v>
       </c>
     </row>
@@ -13344,186 +13532,217 @@
         <v>49.700000000000003</v>
       </c>
       <c r="K2" s="0">
-        <v>0.79598994477964102</v>
+        <v>0.79589292463779804</v>
       </c>
       <c r="L2" s="0">
-        <v>483.96188642602198</v>
+        <v>483.902898179781</v>
       </c>
       <c r="M2" s="0">
-        <v>18.2062582118464</v>
+        <v>18.188120759250801</v>
       </c>
       <c r="N2" s="0">
-        <v>136.245223115523</v>
+        <v>136.25159561144099</v>
       </c>
       <c r="O2" s="0">
-        <v>61.7074477785523</v>
+        <v>61.785965793516397</v>
       </c>
       <c r="P2" s="0">
-        <v>-178.762725371378</v>
+        <v>-270.50944365657603</v>
       </c>
       <c r="Q2" s="0">
-        <v>278.47011357397798</v>
+        <v>278.52910182021901</v>
       </c>
       <c r="R2" s="0">
-        <v>124.719181265611</v>
+        <v>215.75843057441401</v>
       </c>
       <c r="S2" s="0">
-        <v>330.37060526147798</v>
+        <v>331.07910233052098</v>
       </c>
       <c r="T2" s="0">
-        <v>2.14305241826627</v>
+        <v>2.2010125718598998</v>
       </c>
       <c r="U2" s="0">
+        <v>3.10666829816219</v>
+      </c>
+      <c r="V2" s="0">
         <v>3.1105806939880698</v>
       </c>
-      <c r="V2" s="0">
-        <v>0.0010710349999999999</v>
-      </c>
       <c r="W2" s="0">
-        <v>0</v>
+        <v>3.1015983968255401</v>
       </c>
       <c r="X2" s="0">
-        <v>0.00069057034179125399</v>
+        <v>3.1105806939880698</v>
       </c>
       <c r="Y2" s="0">
-        <v>0</v>
+        <v>0.0089822971625248497</v>
       </c>
       <c r="Z2" s="0">
-        <v>0</v>
+        <v>0.00072449884803341504</v>
       </c>
       <c r="AA2" s="0">
+        <v>0.00072541124871377399</v>
+      </c>
+      <c r="AB2" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC2" s="0">
+        <v>0.00022255695558270899</v>
+      </c>
+      <c r="AD2" s="0">
+        <v>0.0146302929715887</v>
+      </c>
+      <c r="AE2" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF2" s="0">
+        <v>0.0010710350000000101</v>
+      </c>
+      <c r="AG2" s="0">
+        <v>0</v>
+      </c>
+      <c r="AH2" s="0">
+        <v>0.00068982910803678599</v>
+      </c>
+      <c r="AI2" s="0">
+        <v>0</v>
+      </c>
+      <c r="AJ2" s="0">
+        <v>0</v>
+      </c>
+      <c r="AK2" s="0">
         <v>3000</v>
       </c>
-      <c r="AB2" s="0">
+      <c r="AL2" s="0">
         <v>57.049944099939403</v>
       </c>
-      <c r="AC2" s="0">
-        <v>29</v>
-      </c>
-      <c r="AD2" s="0">
+      <c r="AM2" s="0">
+        <v>28.9999999999993</v>
+      </c>
+      <c r="AN2" s="0">
         <v>1.2581793901624701</v>
       </c>
-      <c r="AE2" s="0">
-        <v>39.096380864711598</v>
-      </c>
-      <c r="AF2" s="0">
-        <v>1</v>
-      </c>
-      <c r="AG2" s="0">
+      <c r="AO2" s="0">
+        <v>39.096380864711698</v>
+      </c>
+      <c r="AP2" s="0">
+        <v>1</v>
+      </c>
+      <c r="AQ2" s="0">
         <v>112.325</v>
       </c>
-      <c r="AH2" s="0">
-        <v>58.899999999999999</v>
-      </c>
-      <c r="AI2" s="0">
+      <c r="AR2" s="0">
+        <v>58.899999999999899</v>
+      </c>
+      <c r="AS2" s="0">
         <v>141.32499999999999</v>
       </c>
-      <c r="AJ2" s="0">
-        <v>95.221755598253793</v>
-      </c>
-      <c r="AK2" s="0">
-        <v>58.899999999999999</v>
-      </c>
-      <c r="AL2" s="0">
+      <c r="AT2" s="0">
+        <v>95.221755598253395</v>
+      </c>
+      <c r="AU2" s="0">
+        <v>58.899999999999899</v>
+      </c>
+      <c r="AV2" s="0">
         <v>141.32499999999999</v>
       </c>
-      <c r="AM2" s="0">
+      <c r="AW2" s="0">
         <v>0.18702532195876601</v>
       </c>
-      <c r="AN2" s="0">
-        <v>26.431353625822599</v>
-      </c>
-      <c r="AO2" s="0">
-        <v>0.80000000000000004</v>
-      </c>
-      <c r="AP2" s="0">
-        <v>64.707447778552293</v>
-      </c>
-      <c r="AQ2" s="0">
-        <v>0</v>
-      </c>
-      <c r="AR2" s="0">
+      <c r="AX2" s="0">
+        <v>26.431353625822499</v>
+      </c>
+      <c r="AY2" s="0">
+        <v>0.80000000000000204</v>
+      </c>
+      <c r="AZ2" s="0">
+        <v>64.785965793516397</v>
+      </c>
+      <c r="BA2" s="0">
+        <v>0</v>
+      </c>
+      <c r="BB2" s="0">
         <v>5.5</v>
       </c>
-      <c r="AS2" s="0">
+      <c r="BC2" s="0">
         <v>61.600000000000001</v>
       </c>
-      <c r="AT2" s="0">
+      <c r="BD2" s="0">
         <v>60.600000000000001</v>
       </c>
-      <c r="AU2" s="0">
-        <v>1160.7422968259</v>
-      </c>
-      <c r="AV2" s="0" t="s">
+      <c r="BE2" s="0">
+        <v>1160.2049306737599</v>
+      </c>
+      <c r="BF2" s="0" t="s">
         <v>85</v>
       </c>
-      <c r="AW2" s="0" t="s">
+      <c r="BG2" s="0" t="s">
         <v>88</v>
       </c>
-      <c r="AX2" s="0" t="s">
+      <c r="BH2" s="0" t="s">
         <v>90</v>
       </c>
-      <c r="AY2" s="0">
+      <c r="BI2" s="0">
         <v>0.10000000000000001</v>
       </c>
-      <c r="AZ2" s="0">
-        <v>26.431353625822599</v>
-      </c>
-      <c r="BA2" s="0">
-        <v>26.431353625822599</v>
-      </c>
-      <c r="BB2" s="0">
-        <v>0</v>
-      </c>
-      <c r="BC2" s="0">
-        <v>0</v>
-      </c>
-      <c r="BD2" s="0">
-        <v>1</v>
-      </c>
-      <c r="BE2" s="0">
+      <c r="BJ2" s="0">
+        <v>26.431353625822499</v>
+      </c>
+      <c r="BK2" s="0">
+        <v>26.431353625822499</v>
+      </c>
+      <c r="BL2" s="0">
+        <v>0</v>
+      </c>
+      <c r="BM2" s="0">
+        <v>0</v>
+      </c>
+      <c r="BN2" s="0">
+        <v>1</v>
+      </c>
+      <c r="BO2" s="0">
         <v>80</v>
       </c>
-      <c r="BF2" s="0">
+      <c r="BP2" s="0">
         <v>450</v>
       </c>
-      <c r="BG2" s="0">
-        <v>0</v>
-      </c>
-      <c r="BH2" s="0" t="s">
-        <v>98</v>
-      </c>
-      <c r="BI2" s="0" t="s">
+      <c r="BQ2" s="0">
+        <v>0</v>
+      </c>
+      <c r="BR2" s="0" t="s">
+        <v>189</v>
+      </c>
+      <c r="BS2" s="0" t="s">
         <v>81</v>
       </c>
-      <c r="BJ2" s="0" t="s">
+      <c r="BT2" s="0">
+        <v>1</v>
+      </c>
+      <c r="BU2" s="0">
+        <v>1</v>
+      </c>
+      <c r="BV2" s="0">
+        <v>1</v>
+      </c>
+      <c r="BW2" s="0">
+        <v>1</v>
+      </c>
+      <c r="BX2" s="0">
+        <v>0</v>
+      </c>
+      <c r="BY2" s="0"/>
+      <c r="BZ2" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="BK2" s="0">
-        <v>1</v>
-      </c>
-      <c r="BL2" s="0">
-        <v>1</v>
-      </c>
-      <c r="BM2" s="0">
-        <v>1</v>
-      </c>
-      <c r="BN2" s="0">
-        <v>1</v>
-      </c>
-      <c r="BO2" s="0">
-        <v>0</v>
-      </c>
-      <c r="BP2" s="0">
-        <v>0</v>
-      </c>
-      <c r="BQ2" s="0">
-        <v>0</v>
-      </c>
-      <c r="BR2" s="0" t="s">
+      <c r="CA2" s="0">
+        <v>0</v>
+      </c>
+      <c r="CB2" s="0">
+        <v>0</v>
+      </c>
+      <c r="CC2" s="0" t="s">
         <v>103</v>
       </c>
-      <c r="BS2" s="0" t="s">
+      <c r="CD2" s="0" t="s">
         <v>103</v>
       </c>
     </row>
@@ -13553,193 +13772,226 @@
         <v>0.25</v>
       </c>
       <c r="I3" s="0">
-        <v>4</v>
+        <v>1.5</v>
       </c>
       <c r="J3" s="0">
-        <v>198.80000000000001</v>
+        <v>74.549999999999997</v>
       </c>
       <c r="K3" s="0">
-        <v>0.79557081598229196</v>
+        <v>0.79601884289027403</v>
       </c>
       <c r="L3" s="0">
-        <v>483.707056117234</v>
+        <v>483.97945647728602</v>
       </c>
       <c r="M3" s="0">
-        <v>22.398255742957101</v>
+        <v>18.303543395043299</v>
       </c>
       <c r="N3" s="0">
-        <v>137.29828767804099</v>
+        <v>136.901586218311</v>
       </c>
       <c r="O3" s="0">
-        <v>61.7023222830789</v>
+        <v>61.785647303741399</v>
       </c>
       <c r="P3" s="0">
-        <v>-171.70871547189699</v>
+        <v>-270.49731446871101</v>
       </c>
       <c r="Q3" s="0">
-        <v>278.72494388276601</v>
+        <v>278.452543522714</v>
       </c>
       <c r="R3" s="0">
-        <v>118.77358831762901</v>
+        <v>215.39007659484599</v>
       </c>
       <c r="S3" s="0">
-        <v>330.32433472202001</v>
+        <v>331.076235679962</v>
       </c>
       <c r="T3" s="0">
-        <v>1.3357363150150501</v>
+        <v>2.4835457166162</v>
       </c>
       <c r="U3" s="0">
-        <v>0</v>
+        <v>3.3904721939556102</v>
       </c>
       <c r="V3" s="0">
-        <v>0.0042841399999999996</v>
+        <v>3.3950422750398701</v>
       </c>
       <c r="W3" s="0">
-        <v>0.00010420332401484</v>
+        <v>3.38454953876855</v>
       </c>
       <c r="X3" s="0">
-        <v>0.00031260997204452</v>
+        <v>3.3950422750398701</v>
       </c>
       <c r="Y3" s="0">
-        <v>0.00010420332401484</v>
+        <v>0.0104927362713165</v>
       </c>
       <c r="Z3" s="0">
+        <v>0.00081944965274488905</v>
+      </c>
+      <c r="AA3" s="0">
+        <v>0.000820533455065834</v>
+      </c>
+      <c r="AB3" s="0">
+        <v>1</v>
+      </c>
+      <c r="AC3" s="0">
+        <v>0.00022215152250471001</v>
+      </c>
+      <c r="AD3" s="0">
+        <v>0.010752194039667999</v>
+      </c>
+      <c r="AE3" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF3" s="0">
+        <v>0.0016065525</v>
+      </c>
+      <c r="AG3" s="0">
+        <v>0.00019576000595916601</v>
+      </c>
+      <c r="AH3" s="0">
+        <v>0.00058728001787749899</v>
+      </c>
+      <c r="AI3" s="0">
+        <v>0.00019576000595916601</v>
+      </c>
+      <c r="AJ3" s="0">
         <v>0.25</v>
       </c>
-      <c r="AA3" s="0">
-        <v>4000</v>
-      </c>
-      <c r="AB3" s="0">
-        <v>229.267597978629</v>
-      </c>
-      <c r="AC3" s="0">
-        <v>32.304930151602797</v>
-      </c>
-      <c r="AD3" s="0">
-        <v>1.28760231606145</v>
-      </c>
-      <c r="AE3" s="0">
-        <v>173.355840537554</v>
-      </c>
-      <c r="AF3" s="0">
-        <v>0</v>
-      </c>
-      <c r="AG3" s="0">
+      <c r="AK3" s="0">
+        <v>3000</v>
+      </c>
+      <c r="AL3" s="0">
+        <v>85.978742719158006</v>
+      </c>
+      <c r="AM3" s="0">
+        <v>28.402125726489501</v>
+      </c>
+      <c r="AN3" s="0">
+        <v>1.2528566724067101</v>
+      </c>
+      <c r="AO3" s="0">
+        <v>57.651064590146099</v>
+      </c>
+      <c r="AP3" s="0">
+        <v>0</v>
+      </c>
+      <c r="AQ3" s="0">
         <v>112.325</v>
       </c>
-      <c r="AH3" s="0">
-        <v>60.157562130407598</v>
-      </c>
-      <c r="AI3" s="0">
-        <v>144.62993015160299</v>
-      </c>
-      <c r="AJ3" s="0">
-        <v>100.42080601814401</v>
-      </c>
-      <c r="AK3" s="0">
-        <v>58.899999999999999</v>
-      </c>
-      <c r="AL3" s="0">
-        <v>144.62993015160299</v>
-      </c>
-      <c r="AM3" s="0">
-        <v>0.18330727740556099</v>
-      </c>
-      <c r="AN3" s="0">
-        <v>26.511718727446699</v>
-      </c>
-      <c r="AO3" s="0">
-        <v>0.82616402847375803</v>
-      </c>
-      <c r="AP3" s="0">
-        <v>64.7023222830789</v>
-      </c>
-      <c r="AQ3" s="0">
-        <v>0</v>
-      </c>
       <c r="AR3" s="0">
+        <v>59.617233827077101</v>
+      </c>
+      <c r="AS3" s="0">
+        <v>140.72712572648999</v>
+      </c>
+      <c r="AT3" s="0">
+        <v>95.323656967436904</v>
+      </c>
+      <c r="AU3" s="0">
+        <v>58.899999999999899</v>
+      </c>
+      <c r="AV3" s="0">
+        <v>140.72712572648999</v>
+      </c>
+      <c r="AW3" s="0">
+        <v>0.18000045127343001</v>
+      </c>
+      <c r="AX3" s="0">
+        <v>25.330946137181002</v>
+      </c>
+      <c r="AY3" s="0">
+        <v>0.82819841732794497</v>
+      </c>
+      <c r="AZ3" s="0">
+        <v>64.785647303741399</v>
+      </c>
+      <c r="BA3" s="0">
+        <v>0</v>
+      </c>
+      <c r="BB3" s="0">
         <v>5.5</v>
       </c>
-      <c r="AS3" s="0">
+      <c r="BC3" s="0">
         <v>61.600000000000001</v>
       </c>
-      <c r="AT3" s="0">
+      <c r="BD3" s="0">
         <v>60.600000000000001</v>
       </c>
-      <c r="AU3" s="0">
-        <v>1160.7793018652201</v>
-      </c>
-      <c r="AV3" s="0" t="s">
-        <v>86</v>
-      </c>
-      <c r="AW3" s="0" t="s">
-        <v>89</v>
-      </c>
-      <c r="AX3" s="0" t="s">
+      <c r="BE3" s="0">
+        <v>1160.21117599884</v>
+      </c>
+      <c r="BF3" s="0" t="s">
+        <v>187</v>
+      </c>
+      <c r="BG3" s="0" t="s">
+        <v>188</v>
+      </c>
+      <c r="BH3" s="0" t="s">
         <v>90</v>
       </c>
-      <c r="AY3" s="0">
+      <c r="BI3" s="0">
         <v>0.10000000000000001</v>
       </c>
-      <c r="AZ3" s="0">
-        <v>26.431353625822599</v>
-      </c>
-      <c r="BA3" s="0">
-        <v>26.431353625822599</v>
-      </c>
-      <c r="BB3" s="0">
-        <v>0.080365101624163798</v>
-      </c>
-      <c r="BC3" s="0">
-        <v>0.080365101624163798</v>
-      </c>
-      <c r="BD3" s="0">
-        <v>1</v>
-      </c>
-      <c r="BE3" s="0">
-        <v>170</v>
-      </c>
-      <c r="BF3" s="0">
-        <v>590</v>
-      </c>
-      <c r="BG3" s="0">
-        <v>1</v>
-      </c>
-      <c r="BH3" s="0" t="s">
-        <v>98</v>
-      </c>
-      <c r="BI3" s="0" t="s">
-        <v>81</v>
-      </c>
-      <c r="BJ3" s="0" t="s">
+      <c r="BJ3" s="0">
+        <v>26.431353625822499</v>
+      </c>
+      <c r="BK3" s="0">
+        <v>26.431353625822499</v>
+      </c>
+      <c r="BL3" s="0">
+        <v>-1.10040748864155</v>
+      </c>
+      <c r="BM3" s="0">
+        <v>1.10040748864155</v>
+      </c>
+      <c r="BN3" s="0">
+        <v>1</v>
+      </c>
+      <c r="BO3" s="0">
+        <v>80</v>
+      </c>
+      <c r="BP3" s="0">
+        <v>450</v>
+      </c>
+      <c r="BQ3" s="0">
+        <v>1</v>
+      </c>
+      <c r="BR3" s="0" t="s">
+        <v>189</v>
+      </c>
+      <c r="BS3" s="0" t="s">
+        <v>182</v>
+      </c>
+      <c r="BT3" s="0">
+        <v>1</v>
+      </c>
+      <c r="BU3" s="0">
+        <v>1</v>
+      </c>
+      <c r="BV3" s="0">
+        <v>0</v>
+      </c>
+      <c r="BW3" s="0">
+        <v>1</v>
+      </c>
+      <c r="BX3" s="0">
+        <v>1</v>
+      </c>
+      <c r="BY3" s="0">
+        <v>1.1304074886415501</v>
+      </c>
+      <c r="BZ3" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="BK3" s="0">
-        <v>1</v>
-      </c>
-      <c r="BL3" s="0">
-        <v>0</v>
-      </c>
-      <c r="BM3" s="0">
-        <v>1</v>
-      </c>
-      <c r="BN3" s="0">
-        <v>1</v>
-      </c>
-      <c r="BO3" s="0">
-        <v>1</v>
-      </c>
-      <c r="BP3" s="0">
-        <v>1</v>
-      </c>
-      <c r="BQ3" s="0">
-        <v>0</v>
-      </c>
-      <c r="BR3" s="0" t="s">
-        <v>104</v>
-      </c>
-      <c r="BS3" s="0" t="s">
-        <v>104</v>
+      <c r="CA3" s="0">
+        <v>1</v>
+      </c>
+      <c r="CB3" s="0">
+        <v>0</v>
+      </c>
+      <c r="CC3" s="0" t="s">
+        <v>191</v>
+      </c>
+      <c r="CD3" s="0" t="s">
+        <v>191</v>
       </c>
     </row>
   </sheetData>
@@ -13866,10 +14118,10 @@
         <v>57.049944099939403</v>
       </c>
       <c r="H2" s="0">
-        <v>29</v>
+        <v>28.9999999999993</v>
       </c>
       <c r="I2" s="0">
-        <v>39.096380864711598</v>
+        <v>39.096380864711698</v>
       </c>
       <c r="J2" s="0">
         <v>0</v>
@@ -13878,31 +14130,31 @@
         <v>0.18702532195876601</v>
       </c>
       <c r="L2" s="0">
-        <v>26.431353625822599</v>
+        <v>26.431353625822499</v>
       </c>
       <c r="M2" s="0">
         <v>0</v>
       </c>
       <c r="N2" s="0">
-        <v>0.79598994477964102</v>
+        <v>0.79589292463779804</v>
       </c>
       <c r="O2" s="0">
         <v>0</v>
       </c>
       <c r="P2" s="0">
-        <v>483.96188642602198</v>
+        <v>483.902898179781</v>
       </c>
       <c r="Q2" s="0">
         <v>0</v>
       </c>
       <c r="R2" s="0">
-        <v>3.1105806939880698</v>
+        <v>3.10666829816219</v>
       </c>
       <c r="S2" s="0">
-        <v>0.80000000000000004</v>
+        <v>0.80000000000000204</v>
       </c>
       <c r="T2" s="0">
-        <v>61.7074477785523</v>
+        <v>61.785965793516397</v>
       </c>
       <c r="U2" s="0" t="s">
         <v>103</v>
@@ -13913,7 +14165,7 @@
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>86</v>
+        <v>187</v>
       </c>
       <c r="B3" s="0">
         <v>0.10000000000000001</v>
@@ -13922,58 +14174,58 @@
         <v>0.25</v>
       </c>
       <c r="D3" s="0">
-        <v>4</v>
+        <v>1.5</v>
       </c>
       <c r="E3" s="0">
-        <v>198.80000000000001</v>
+        <v>74.549999999999997</v>
       </c>
       <c r="F3" s="0">
-        <v>4000</v>
+        <v>3000</v>
       </c>
       <c r="G3" s="0">
-        <v>229.267597978629</v>
+        <v>85.978742719158006</v>
       </c>
       <c r="H3" s="0">
-        <v>32.304930151602797</v>
+        <v>28.402125726489501</v>
       </c>
       <c r="I3" s="0">
-        <v>173.355840537554</v>
+        <v>57.651064590146099</v>
       </c>
       <c r="J3" s="0">
         <v>1</v>
       </c>
       <c r="K3" s="0">
-        <v>0.18330727740556099</v>
+        <v>0.18000045127343001</v>
       </c>
       <c r="L3" s="0">
-        <v>26.511718727446699</v>
+        <v>25.330946137181002</v>
       </c>
       <c r="M3" s="0">
-        <v>0.080365101624163798</v>
+        <v>-1.10040748864155</v>
       </c>
       <c r="N3" s="0">
-        <v>0.79557081598229196</v>
+        <v>0.79601884289027403</v>
       </c>
       <c r="O3" s="0">
-        <v>-0.00041912879734917801</v>
+        <v>0.00012591825247632</v>
       </c>
       <c r="P3" s="0">
-        <v>483.707056117234</v>
+        <v>483.97945647728602</v>
       </c>
       <c r="Q3" s="0">
-        <v>-0.25483030878825702</v>
+        <v>0.0765582975052439</v>
       </c>
       <c r="R3" s="0">
-        <v>0</v>
+        <v>3.3904721939556102</v>
       </c>
       <c r="S3" s="0">
-        <v>0.82616402847375803</v>
+        <v>0.82819841732794497</v>
       </c>
       <c r="T3" s="0">
-        <v>61.7023222830789</v>
+        <v>61.785647303741399</v>
       </c>
       <c r="U3" s="0" t="s">
-        <v>104</v>
+        <v>191</v>
       </c>
       <c r="V3" s="0">
         <v>0</v>
@@ -14014,7 +14266,7 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>146</v>
+        <v>193</v>
       </c>
       <c r="B2" s="0" t="s">
         <v>114</v>
@@ -14027,6 +14279,1239 @@
       </c>
       <c r="E2" s="0" t="s">
         <v>120</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:P14"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="10" customWidth="true"/>
+    <col min="2" max="2" width="11" customWidth="true"/>
+    <col min="3" max="3" width="9" customWidth="true"/>
+    <col min="4" max="4" width="20.21875" customWidth="true"/>
+    <col min="5" max="5" width="11.77734375" customWidth="true"/>
+    <col min="6" max="6" width="12.5546875" customWidth="true"/>
+    <col min="7" max="7" width="12.109375" customWidth="true"/>
+    <col min="8" max="8" width="11.5546875" customWidth="true"/>
+    <col min="9" max="9" width="25.6640625" customWidth="true"/>
+    <col min="10" max="10" width="11.5546875" customWidth="true"/>
+    <col min="11" max="11" width="11" customWidth="true"/>
+    <col min="12" max="12" width="12.5546875" customWidth="true"/>
+    <col min="13" max="13" width="16.21875" customWidth="true"/>
+    <col min="14" max="14" width="13.21875" customWidth="true"/>
+    <col min="15" max="15" width="15.21875" customWidth="true"/>
+    <col min="16" max="16" width="15.21875" customWidth="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="0" t="s">
+        <v>147</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>105</v>
+      </c>
+      <c r="E1" s="0" t="s">
+        <v>158</v>
+      </c>
+      <c r="F1" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G1" s="0" t="s">
+        <v>159</v>
+      </c>
+      <c r="H1" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1" s="0" t="s">
+        <v>160</v>
+      </c>
+      <c r="J1" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="K1" s="0" t="s">
+        <v>161</v>
+      </c>
+      <c r="L1" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="M1" s="0" t="s">
+        <v>162</v>
+      </c>
+      <c r="N1" s="0" t="s">
+        <v>163</v>
+      </c>
+      <c r="O1" s="0" t="s">
+        <v>164</v>
+      </c>
+      <c r="P1" s="0" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="0">
+        <v>38</v>
+      </c>
+      <c r="D2" s="0">
+        <v>0.10000000000000001</v>
+      </c>
+      <c r="E2" s="0">
+        <v>0.80169999999999997</v>
+      </c>
+      <c r="F2" s="0">
+        <v>0.79598994477964102</v>
+      </c>
+      <c r="G2" s="0">
+        <v>53</v>
+      </c>
+      <c r="H2" s="0">
+        <v>61.7074477785523</v>
+      </c>
+      <c r="I2" s="0">
+        <v>141.32499999999999</v>
+      </c>
+      <c r="J2" s="0">
+        <v>141.32499999999999</v>
+      </c>
+      <c r="K2" s="0">
+        <v>0.80000000000000004</v>
+      </c>
+      <c r="L2" s="0">
+        <v>0.80000000000000004</v>
+      </c>
+      <c r="M2" s="0">
+        <v>-0.005710055220358945</v>
+      </c>
+      <c r="N2" s="0">
+        <v>8.7074477785523001</v>
+      </c>
+      <c r="O2" s="0">
+        <v>0</v>
+      </c>
+      <c r="P2" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="0">
+        <v>76</v>
+      </c>
+      <c r="D3" s="0">
+        <v>0.20000000000000001</v>
+      </c>
+      <c r="E3" s="0">
+        <v>0.77259999999999995</v>
+      </c>
+      <c r="F3" s="0">
+        <v>0.77368670273936202</v>
+      </c>
+      <c r="G3" s="0">
+        <v>59.299999999999997</v>
+      </c>
+      <c r="H3" s="0">
+        <v>63.474856572649799</v>
+      </c>
+      <c r="I3" s="0">
+        <v>156.225</v>
+      </c>
+      <c r="J3" s="0">
+        <v>156.225</v>
+      </c>
+      <c r="K3" s="0">
+        <v>0.59999999999999998</v>
+      </c>
+      <c r="L3" s="0">
+        <v>0.59999999999999998</v>
+      </c>
+      <c r="M3" s="0">
+        <v>0.0010867027393620665</v>
+      </c>
+      <c r="N3" s="0">
+        <v>4.1748565726498015</v>
+      </c>
+      <c r="O3" s="0">
+        <v>0</v>
+      </c>
+      <c r="P3" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="0">
+        <v>114</v>
+      </c>
+      <c r="D4" s="0">
+        <v>0.29999999999999999</v>
+      </c>
+      <c r="E4" s="0">
+        <v>0.75039999999999996</v>
+      </c>
+      <c r="F4" s="0">
+        <v>0.75754557689535296</v>
+      </c>
+      <c r="G4" s="0">
+        <v>61.399999999999999</v>
+      </c>
+      <c r="H4" s="0">
+        <v>64.875151556498693</v>
+      </c>
+      <c r="I4" s="0">
+        <v>161.32499999999999</v>
+      </c>
+      <c r="J4" s="0">
+        <v>161.32500000421999</v>
+      </c>
+      <c r="K4" s="0">
+        <v>0.59999999999999998</v>
+      </c>
+      <c r="L4" s="0">
+        <v>0.60000000001569298</v>
+      </c>
+      <c r="M4" s="0">
+        <v>0.0071455768953530008</v>
+      </c>
+      <c r="N4" s="0">
+        <v>3.4751515564986946</v>
+      </c>
+      <c r="O4" s="0">
+        <v>4.2199985728075262e-09</v>
+      </c>
+      <c r="P4" s="0">
+        <v>1.5693002453076588e-11</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>148</v>
+      </c>
+      <c r="C5" s="0">
+        <v>152</v>
+      </c>
+      <c r="D5" s="0">
+        <v>0.40000000000000002</v>
+      </c>
+      <c r="E5" s="0">
+        <v>0.73380000000000001</v>
+      </c>
+      <c r="F5" s="0">
+        <v>0.74303041406938997</v>
+      </c>
+      <c r="G5" s="0">
+        <v>64.5</v>
+      </c>
+      <c r="H5" s="0">
+        <v>66.5729018811831</v>
+      </c>
+      <c r="I5" s="0">
+        <v>171.42500000000001</v>
+      </c>
+      <c r="J5" s="0">
+        <v>171.42500000251999</v>
+      </c>
+      <c r="K5" s="0">
+        <v>0.59999999999999998</v>
+      </c>
+      <c r="L5" s="0">
+        <v>0.60000000000882103</v>
+      </c>
+      <c r="M5" s="0">
+        <v>0.0092304140693899584</v>
+      </c>
+      <c r="N5" s="0">
+        <v>2.0729018811830997</v>
+      </c>
+      <c r="O5" s="0">
+        <v>2.5199824449373409e-09</v>
+      </c>
+      <c r="P5" s="0">
+        <v>8.8210549975542563e-12</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>149</v>
+      </c>
+      <c r="C6" s="0">
+        <v>228</v>
+      </c>
+      <c r="D6" s="0">
+        <v>0.59999999999999998</v>
+      </c>
+      <c r="E6" s="0">
+        <v>0.71020000000000005</v>
+      </c>
+      <c r="F6" s="0">
+        <v>0.71577815827091795</v>
+      </c>
+      <c r="G6" s="0">
+        <v>70.700000000000003</v>
+      </c>
+      <c r="H6" s="0">
+        <v>71.333508647832602</v>
+      </c>
+      <c r="I6" s="0">
+        <v>191.32499999999999</v>
+      </c>
+      <c r="J6" s="0">
+        <v>191.32500000246401</v>
+      </c>
+      <c r="K6" s="0">
+        <v>0.59999999999999998</v>
+      </c>
+      <c r="L6" s="0">
+        <v>0.60000000000772702</v>
+      </c>
+      <c r="M6" s="0">
+        <v>0.005578158270917899</v>
+      </c>
+      <c r="N6" s="0">
+        <v>0.63350864783259908</v>
+      </c>
+      <c r="O6" s="0">
+        <v>2.4640200990688754e-09</v>
+      </c>
+      <c r="P6" s="0">
+        <v>7.727041229088627e-12</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>150</v>
+      </c>
+      <c r="C7" s="0">
+        <v>266</v>
+      </c>
+      <c r="D7" s="0">
+        <v>0.69999999999999996</v>
+      </c>
+      <c r="E7" s="0">
+        <v>0.70120000000000005</v>
+      </c>
+      <c r="F7" s="0">
+        <v>0.70199027041918405</v>
+      </c>
+      <c r="G7" s="0">
+        <v>74.099999999999994</v>
+      </c>
+      <c r="H7" s="0">
+        <v>74.3989051619061</v>
+      </c>
+      <c r="I7" s="0">
+        <v>201.32499999999999</v>
+      </c>
+      <c r="J7" s="0">
+        <v>201.32500000222899</v>
+      </c>
+      <c r="K7" s="0">
+        <v>0.59999999999999998</v>
+      </c>
+      <c r="L7" s="0">
+        <v>0.600000000006642</v>
+      </c>
+      <c r="M7" s="0">
+        <v>0.00079027041918400265</v>
+      </c>
+      <c r="N7" s="0">
+        <v>0.29890516190610583</v>
+      </c>
+      <c r="O7" s="0">
+        <v>2.2290009837888647e-09</v>
+      </c>
+      <c r="P7" s="0">
+        <v>6.6420202671224615e-12</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0" t="s">
+        <v>151</v>
+      </c>
+      <c r="C8" s="0">
+        <v>342</v>
+      </c>
+      <c r="D8" s="0">
+        <v>0.90000000000000002</v>
+      </c>
+      <c r="E8" s="0">
+        <v>0.68259999999999999</v>
+      </c>
+      <c r="F8" s="0">
+        <v>0.68257303198983999</v>
+      </c>
+      <c r="G8" s="0">
+        <v>77.5</v>
+      </c>
+      <c r="H8" s="0">
+        <v>76.267066152398101</v>
+      </c>
+      <c r="I8" s="0">
+        <v>221.32499999999999</v>
+      </c>
+      <c r="J8" s="0">
+        <v>221.32500000182401</v>
+      </c>
+      <c r="K8" s="0">
+        <v>0.59999999999999998</v>
+      </c>
+      <c r="L8" s="0">
+        <v>0.60000000000494602</v>
+      </c>
+      <c r="M8" s="0">
+        <v>-2.6968010160000055e-05</v>
+      </c>
+      <c r="N8" s="0">
+        <v>-1.2329338476018989</v>
+      </c>
+      <c r="O8" s="0">
+        <v>1.824020046115038e-09</v>
+      </c>
+      <c r="P8" s="0">
+        <v>4.9460435747050724e-12</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="C9" s="0">
+        <v>418</v>
+      </c>
+      <c r="D9" s="0">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="E9" s="0">
+        <v>0.66600000000000004</v>
+      </c>
+      <c r="F9" s="0">
+        <v>0.66463990247187399</v>
+      </c>
+      <c r="G9" s="0">
+        <v>78.799999999999997</v>
+      </c>
+      <c r="H9" s="0">
+        <v>77.593739480074703</v>
+      </c>
+      <c r="I9" s="0">
+        <v>241.32499999999999</v>
+      </c>
+      <c r="J9" s="0">
+        <v>241.32500000019201</v>
+      </c>
+      <c r="K9" s="0">
+        <v>0.59999999999999998</v>
+      </c>
+      <c r="L9" s="0">
+        <v>0.60000000000047704</v>
+      </c>
+      <c r="M9" s="0">
+        <v>-0.0013600975281260475</v>
+      </c>
+      <c r="N9" s="0">
+        <v>-1.2062605199252943</v>
+      </c>
+      <c r="O9" s="0">
+        <v>1.9201706891180947e-10</v>
+      </c>
+      <c r="P9" s="0">
+        <v>4.7706283368142977e-13</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0" t="s">
+        <v>153</v>
+      </c>
+      <c r="C10" s="0">
+        <v>494</v>
+      </c>
+      <c r="D10" s="0">
+        <v>1.3</v>
+      </c>
+      <c r="E10" s="0">
+        <v>0.64690000000000003</v>
+      </c>
+      <c r="F10" s="0">
+        <v>0.64634780467543396</v>
+      </c>
+      <c r="G10" s="0">
+        <v>79.599999999999994</v>
+      </c>
+      <c r="H10" s="0">
+        <v>78.789912798525506</v>
+      </c>
+      <c r="I10" s="0">
+        <v>251.32499999999999</v>
+      </c>
+      <c r="J10" s="0">
+        <v>251.325000000241</v>
+      </c>
+      <c r="K10" s="0">
+        <v>0.5</v>
+      </c>
+      <c r="L10" s="0">
+        <v>0.50000000000047895</v>
+      </c>
+      <c r="M10" s="0">
+        <v>-0.00055219532456607379</v>
+      </c>
+      <c r="N10" s="0">
+        <v>-0.81008720147448798</v>
+      </c>
+      <c r="O10" s="0">
+        <v>2.4101609596982598e-10</v>
+      </c>
+      <c r="P10" s="0">
+        <v>4.7895021282329253e-13</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0" t="s">
+        <v>154</v>
+      </c>
+      <c r="C11" s="0">
+        <v>570</v>
+      </c>
+      <c r="D11" s="0">
+        <v>1.5</v>
+      </c>
+      <c r="E11" s="0">
+        <v>0.624</v>
+      </c>
+      <c r="F11" s="0">
+        <v>0.628633964841112</v>
+      </c>
+      <c r="G11" s="0">
+        <v>80.099999999999994</v>
+      </c>
+      <c r="H11" s="0">
+        <v>79.144636855140305</v>
+      </c>
+      <c r="I11" s="0">
+        <v>251.22500000000002</v>
+      </c>
+      <c r="J11" s="0">
+        <v>251.22500000062399</v>
+      </c>
+      <c r="K11" s="0">
+        <v>0.45000000000000001</v>
+      </c>
+      <c r="L11" s="0">
+        <v>0.45000000000111701</v>
+      </c>
+      <c r="M11" s="0">
+        <v>0.0046339648411120038</v>
+      </c>
+      <c r="N11" s="0">
+        <v>-0.95536314485968887</v>
+      </c>
+      <c r="O11" s="0">
+        <v>6.2397020883508958e-10</v>
+      </c>
+      <c r="P11" s="0">
+        <v>1.11699538507537e-12</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0" t="s">
+        <v>155</v>
+      </c>
+      <c r="C12" s="0">
+        <v>646</v>
+      </c>
+      <c r="D12" s="0">
+        <v>1.7</v>
+      </c>
+      <c r="E12" s="0">
+        <v>0.60189999999999999</v>
+      </c>
+      <c r="F12" s="0">
+        <v>0.61102459386595498</v>
+      </c>
+      <c r="G12" s="0">
+        <v>80</v>
+      </c>
+      <c r="H12" s="0">
+        <v>79.503558843833702</v>
+      </c>
+      <c r="I12" s="0">
+        <v>251.42500000000001</v>
+      </c>
+      <c r="J12" s="0">
+        <v>251.42500005294801</v>
+      </c>
+      <c r="K12" s="0">
+        <v>0.40000000000000002</v>
+      </c>
+      <c r="L12" s="0">
+        <v>0.40000000008423697</v>
+      </c>
+      <c r="M12" s="0">
+        <v>0.0091245938659549886</v>
+      </c>
+      <c r="N12" s="0">
+        <v>-0.49644115616629847</v>
+      </c>
+      <c r="O12" s="0">
+        <v>5.2947996209695703e-08</v>
+      </c>
+      <c r="P12" s="0">
+        <v>8.4236950748106665e-11</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0" t="s">
+        <v>156</v>
+      </c>
+      <c r="C13" s="0">
+        <v>684</v>
+      </c>
+      <c r="D13" s="0">
+        <v>1.8</v>
+      </c>
+      <c r="E13" s="0">
+        <v>0.59019999999999995</v>
+      </c>
+      <c r="F13" s="0">
+        <v>0.60218938142780398</v>
+      </c>
+      <c r="G13" s="0">
+        <v>80.200000000000003</v>
+      </c>
+      <c r="H13" s="0">
+        <v>79.603384208279607</v>
+      </c>
+      <c r="I13" s="0">
+        <v>251.22500000000002</v>
+      </c>
+      <c r="J13" s="0">
+        <v>251.225000069309</v>
+      </c>
+      <c r="K13" s="0">
+        <v>0.40000000000000002</v>
+      </c>
+      <c r="L13" s="0">
+        <v>0.40000000011035303</v>
+      </c>
+      <c r="M13" s="0">
+        <v>0.011989381427804036</v>
+      </c>
+      <c r="N13" s="0">
+        <v>-0.5966157917203958</v>
+      </c>
+      <c r="O13" s="0">
+        <v>6.93089816650172e-08</v>
+      </c>
+      <c r="P13" s="0">
+        <v>1.1035300451212038e-10</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0">
+        <v>13</v>
+      </c>
+      <c r="B14" s="0" t="s">
+        <v>157</v>
+      </c>
+      <c r="C14" s="0">
+        <v>722</v>
+      </c>
+      <c r="D14" s="0">
+        <v>1.8999999999999999</v>
+      </c>
+      <c r="E14" s="0">
+        <v>0.57889999999999997</v>
+      </c>
+      <c r="F14" s="0">
+        <v>0.592933152962411</v>
+      </c>
+      <c r="G14" s="0">
+        <v>80.400000000000006</v>
+      </c>
+      <c r="H14" s="0">
+        <v>79.957842632891399</v>
+      </c>
+      <c r="I14" s="0">
+        <v>251.32499999999999</v>
+      </c>
+      <c r="J14" s="0">
+        <v>251.32500008692301</v>
+      </c>
+      <c r="K14" s="0">
+        <v>0.40000000000000002</v>
+      </c>
+      <c r="L14" s="0">
+        <v>0.40000000013834403</v>
+      </c>
+      <c r="M14" s="0">
+        <v>0.014033152962411033</v>
+      </c>
+      <c r="N14" s="0">
+        <v>-0.44215736710860654</v>
+      </c>
+      <c r="O14" s="0">
+        <v>8.6923023445706349e-08</v>
+      </c>
+      <c r="P14" s="0">
+        <v>1.3834400292012106e-10</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="11.21875" customWidth="true"/>
+    <col min="2" max="2" width="15.21875" customWidth="true"/>
+    <col min="3" max="3" width="15.21875" customWidth="true"/>
+    <col min="4" max="4" width="10.88671875" customWidth="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="0" t="s">
+        <v>166</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>167</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>168</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="s">
+        <v>75</v>
+      </c>
+      <c r="B2" s="0">
+        <v>0.0070675196837638871</v>
+      </c>
+      <c r="C2" s="0">
+        <v>0.014033152962411033</v>
+      </c>
+      <c r="D2" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="0">
+        <v>2.9801317725066774</v>
+      </c>
+      <c r="C3" s="0">
+        <v>8.7074477785523001</v>
+      </c>
+      <c r="D3" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="B4" s="0">
+        <v>3.4196094169882921e-08</v>
+      </c>
+      <c r="C4" s="0">
+        <v>8.6923023445706349e-08</v>
+      </c>
+      <c r="D4" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="B5" s="0">
+        <v>5.4678631436356117e-11</v>
+      </c>
+      <c r="C5" s="0">
+        <v>1.3834400292012106e-10</v>
+      </c>
+      <c r="D5" s="0">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:BF2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="8.6640625" customWidth="true"/>
+    <col min="2" max="2" width="7.109375" customWidth="true"/>
+    <col min="3" max="3" width="18.6640625" customWidth="true"/>
+    <col min="4" max="4" width="17.6640625" customWidth="true"/>
+    <col min="5" max="5" width="28.88671875" customWidth="true"/>
+    <col min="6" max="6" width="9" customWidth="true"/>
+    <col min="7" max="7" width="29.33203125" customWidth="true"/>
+    <col min="8" max="8" width="15.44140625" customWidth="true"/>
+    <col min="9" max="9" width="12.88671875" customWidth="true"/>
+    <col min="10" max="10" width="21.77734375" customWidth="true"/>
+    <col min="11" max="11" width="9.6640625" customWidth="true"/>
+    <col min="12" max="12" width="13.77734375" customWidth="true"/>
+    <col min="13" max="13" width="13.44140625" customWidth="true"/>
+    <col min="14" max="14" width="18.33203125" customWidth="true"/>
+    <col min="15" max="15" width="9.33203125" customWidth="true"/>
+    <col min="16" max="16" width="14" customWidth="true"/>
+    <col min="17" max="17" width="9" customWidth="true"/>
+    <col min="18" max="18" width="9.6640625" customWidth="true"/>
+    <col min="19" max="19" width="9.6640625" customWidth="true"/>
+    <col min="20" max="20" width="8.77734375" customWidth="true"/>
+    <col min="21" max="21" width="16.33203125" customWidth="true"/>
+    <col min="22" max="22" width="18.5546875" customWidth="true"/>
+    <col min="23" max="23" width="16.6640625" customWidth="true"/>
+    <col min="24" max="24" width="16.77734375" customWidth="true"/>
+    <col min="25" max="25" width="19.6640625" customWidth="true"/>
+    <col min="26" max="26" width="15.77734375" customWidth="true"/>
+    <col min="27" max="27" width="15" customWidth="true"/>
+    <col min="28" max="28" width="13.6640625" customWidth="true"/>
+    <col min="29" max="29" width="11.88671875" customWidth="true"/>
+    <col min="30" max="30" width="17.77734375" customWidth="true"/>
+    <col min="31" max="31" width="14" customWidth="true"/>
+    <col min="32" max="32" width="22.109375" customWidth="true"/>
+    <col min="33" max="33" width="13.33203125" customWidth="true"/>
+    <col min="34" max="34" width="11.5546875" customWidth="true"/>
+    <col min="35" max="35" width="14.6640625" customWidth="true"/>
+    <col min="36" max="36" width="12.88671875" customWidth="true"/>
+    <col min="37" max="37" width="9.44140625" customWidth="true"/>
+    <col min="38" max="38" width="11.21875" customWidth="true"/>
+    <col min="39" max="39" width="9.5546875" customWidth="true"/>
+    <col min="40" max="40" width="13.5546875" customWidth="true"/>
+    <col min="41" max="41" width="8.6640625" customWidth="true"/>
+    <col min="42" max="42" width="13" customWidth="true"/>
+    <col min="43" max="43" width="23.88671875" customWidth="true"/>
+    <col min="44" max="44" width="17.77734375" customWidth="true"/>
+    <col min="45" max="45" width="19.109375" customWidth="true"/>
+    <col min="46" max="46" width="20.44140625" customWidth="true"/>
+    <col min="47" max="47" width="19.5546875" customWidth="true"/>
+    <col min="48" max="48" width="26.109375" customWidth="true"/>
+    <col min="49" max="49" width="14.6640625" customWidth="true"/>
+    <col min="50" max="50" width="9.88671875" customWidth="true"/>
+    <col min="51" max="51" width="9.77734375" customWidth="true"/>
+    <col min="52" max="52" width="10.33203125" customWidth="true"/>
+    <col min="53" max="53" width="11" customWidth="true"/>
+    <col min="54" max="54" width="16.33203125" customWidth="true"/>
+    <col min="55" max="55" width="12.5546875" customWidth="true"/>
+    <col min="56" max="56" width="18.77734375" customWidth="true"/>
+    <col min="57" max="57" width="8.6640625" customWidth="true"/>
+    <col min="58" max="58" width="18.21875" customWidth="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="I1" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="J1" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="K1" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="L1" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="M1" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="N1" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="O1" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="P1" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q1" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="R1" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="S1" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="T1" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="U1" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="V1" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="W1" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="X1" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z1" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="AA1" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB1" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="AC1" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="AD1" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="AE1" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="AF1" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="AG1" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="AH1" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="AI1" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="AJ1" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="AK1" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="AL1" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="AM1" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="AN1" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="AO1" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="AP1" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="AQ1" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="AR1" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="AS1" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AT1" s="0" t="s">
+        <v>49</v>
+      </c>
+      <c r="AU1" s="0" t="s">
+        <v>50</v>
+      </c>
+      <c r="AV1" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="AW1" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="AX1" s="0" t="s">
+        <v>54</v>
+      </c>
+      <c r="AY1" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="AZ1" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="BA1" s="0" t="s">
+        <v>57</v>
+      </c>
+      <c r="BB1" s="0" t="s">
+        <v>58</v>
+      </c>
+      <c r="BC1" s="0" t="s">
+        <v>59</v>
+      </c>
+      <c r="BD1" s="0" t="s">
+        <v>60</v>
+      </c>
+      <c r="BE1" s="0" t="s">
+        <v>61</v>
+      </c>
+      <c r="BF1" s="0" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="0">
+        <v>1</v>
+      </c>
+      <c r="D2" s="0">
+        <v>38</v>
+      </c>
+      <c r="E2" s="0">
+        <v>0.10000000000000001</v>
+      </c>
+      <c r="F2" s="0">
+        <v>38</v>
+      </c>
+      <c r="G2" s="0">
+        <v>0.10000000000000001</v>
+      </c>
+      <c r="H2" s="0">
+        <v>0.29999999999999999</v>
+      </c>
+      <c r="I2" s="0">
+        <v>1</v>
+      </c>
+      <c r="J2" s="0">
+        <v>49.700000000000003</v>
+      </c>
+      <c r="K2" s="0">
+        <v>0.79532989041314495</v>
+      </c>
+      <c r="L2" s="0">
+        <v>483.56057337119199</v>
+      </c>
+      <c r="M2" s="0">
+        <v>16.598160605899999</v>
+      </c>
+      <c r="N2" s="0">
+        <v>136.11978826018199</v>
+      </c>
+      <c r="O2" s="0">
+        <v>61.7077338870264</v>
+      </c>
+      <c r="P2" s="0">
+        <v>-178.73838162904201</v>
+      </c>
+      <c r="Q2" s="0">
+        <v>278.87142662880802</v>
+      </c>
+      <c r="R2" s="0">
+        <v>125.049993617334</v>
+      </c>
+      <c r="S2" s="0">
+        <v>330.37317975087001</v>
+      </c>
+      <c r="T2" s="0">
+        <v>2.1866348896457</v>
+      </c>
+      <c r="U2" s="0">
+        <v>2.9673537389428901</v>
+      </c>
+      <c r="V2" s="0">
+        <v>0.0010710349999999999</v>
+      </c>
+      <c r="W2" s="0">
+        <v>0.00021157558755779301</v>
+      </c>
+      <c r="X2" s="0">
+        <v>0.00049367637096818398</v>
+      </c>
+      <c r="Y2" s="0">
+        <v>0.00021157558755779301</v>
+      </c>
+      <c r="Z2" s="0">
+        <v>0.29999999999999999</v>
+      </c>
+      <c r="AA2" s="0">
+        <v>3000</v>
+      </c>
+      <c r="AB2" s="0">
+        <v>57.518862405345402</v>
+      </c>
+      <c r="AC2" s="0">
+        <v>29</v>
+      </c>
+      <c r="AD2" s="0">
+        <v>1.2581793901624701</v>
+      </c>
+      <c r="AE2" s="0">
+        <v>39.231472803106001</v>
+      </c>
+      <c r="AF2" s="0">
+        <v>1</v>
+      </c>
+      <c r="AG2" s="0">
+        <v>112.325</v>
+      </c>
+      <c r="AH2" s="0">
+        <v>60.047351165292802</v>
+      </c>
+      <c r="AI2" s="0">
+        <v>141.32499999999999</v>
+      </c>
+      <c r="AJ2" s="0">
+        <v>96.494611382161693</v>
+      </c>
+      <c r="AK2" s="0">
+        <v>58.899999999999999</v>
+      </c>
+      <c r="AL2" s="0">
+        <v>141.32499999999999</v>
+      </c>
+      <c r="AM2" s="0">
+        <v>0.17329139734382101</v>
+      </c>
+      <c r="AN2" s="0">
+        <v>24.490406729615501</v>
+      </c>
+      <c r="AO2" s="0">
+        <v>0.85675983892366803</v>
+      </c>
+      <c r="AP2" s="0">
+        <v>64.707733887026393</v>
+      </c>
+      <c r="AQ2" s="0">
+        <v>0</v>
+      </c>
+      <c r="AR2" s="0">
+        <v>5.5</v>
+      </c>
+      <c r="AS2" s="0">
+        <v>61.600000000000001</v>
+      </c>
+      <c r="AT2" s="0">
+        <v>60.600000000000001</v>
+      </c>
+      <c r="AU2" s="0">
+        <v>1160.7303613460599</v>
+      </c>
+      <c r="AV2" s="0">
+        <v>0.10000000000000001</v>
+      </c>
+      <c r="AW2" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="AX2" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="AY2" s="0">
+        <v>1</v>
+      </c>
+      <c r="AZ2" s="0">
+        <v>1</v>
+      </c>
+      <c r="BA2" s="0">
+        <v>1</v>
+      </c>
+      <c r="BB2" s="0">
+        <v>1</v>
+      </c>
+      <c r="BC2" s="0">
+        <v>0</v>
+      </c>
+      <c r="BD2" s="0">
+        <v>1</v>
+      </c>
+      <c r="BE2" s="0" t="s">
+        <v>62</v>
+      </c>
+      <c r="BF2" s="0" t="s">
+        <v>62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>